<commit_message>
additional solution and MECE update
</commit_message>
<xml_diff>
--- a/MECE/MECE.xlsx
+++ b/MECE/MECE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jange\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AIDS\Group4\MECE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B1C2F0-DBC3-4074-92B3-172A9E784837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5794BF43-B66E-4D65-9690-00789540481C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{968BD888-7518-41E0-AA3A-CCE61A65B882}"/>
   </bookViews>
@@ -58,6 +58,13 @@
   <si>
     <t xml:space="preserve">
 </t>
+  </si>
+  <si>
+    <t>Part 1:
+Q6  What is the total number of ip addresses across all the records?
+Q8  What is the total number of hashtags across all these tweets?
+Part2:
+Q4  What is the change in word frequencies if normalization is done after stop word removal.</t>
   </si>
   <si>
     <r>
@@ -99,21 +106,22 @@
       </rPr>
       <t>).
 Use regular expressions to find both standard and obfuscated IP addresses in the text.
-Count how many total IP addresses appear across all the rows and print the final number.</t>
+Count how many total IP addresses appear across all the rows and print the final number.
+Compare two preprocessing methods:
+Method A: Stopword Removal → then Stemming
+Method B: Stemming → then Stopword Removal
+And analyze how the order of these steps affects the frequency of words in a text dataset.</t>
     </r>
   </si>
   <si>
+    <t>6 -Total unique IP-like matches found: 80
+8-Total number of hashtags across all tweets: 2924
+4-The order of preprocessing steps makes a big difference. Stemming before removing stopwords helps keep more information intact and leads to richer, more reliable data for downstream tasks.</t>
+  </si>
+  <si>
     <t>just check all the possible ways to find the ip and give the regex python code to find them all
-it doesnt has any column it only has one colum and the data is in sentences</t>
-  </si>
-  <si>
-    <t>Total unique IP-like matches found: 80
-Total number of hashtags across all tweets: 2924</t>
-  </si>
-  <si>
-    <t>Part 1:
-Q6  What is the total number of ip addresses across all the records?
-Q8  What is the total number of hashtags across all these tweets?</t>
+it doesnt has any column it only has one colum and the data is in sentences
+is it possible to explain with any visualization?</t>
   </si>
 </sst>
 </file>
@@ -537,21 +545,21 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="86.4">
+    <row r="2" spans="1:5" ht="158.4">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.8">

</xml_diff>